<commit_message>
RP-1048 Journeys J3-J6, J9-J12, J14, the VIS re-run, final results and the rebuilt workbook
All 262 Test Cases and 15 journeys run on current main as every seeded role.
No visibility leak found. Bugs: RP-1049, RP-1050, RP-1051, RP-1052, RP-1053,
RP-1055, RP-1056 (and RP-921 seen again).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/uat/round-0/fixtures-data/bad-rows.xlsx
+++ b/planning/uat/round-0/fixtures-data/bad-rows.xlsx
@@ -30,7 +30,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UAT IMP-04 184405 item 1</t>
+          <t xml:space="preserve">UAT IMP-04 190749 item 1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -59,7 +59,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UAT IMP-04 184405 xxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxx</t>
+          <t xml:space="preserve">UAT IMP-04 190749 xxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -76,7 +76,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">UAT IMP-04 184405 unknown type</t>
+          <t xml:space="preserve">UAT IMP-04 190749 unknown type</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -93,7 +93,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">UAT IMP-04 184405 unknown trade</t>
+          <t xml:space="preserve">UAT IMP-04 190749 unknown trade</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -110,7 +110,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UAT IMP-04 184405 outside visibility</t>
+          <t xml:space="preserve">UAT IMP-04 190749 outside visibility</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>